<commit_message>
Visuel v3: badges club sur la carte, soldes mercato 2026, partenaires FX; donnees Reims L2 / Paris FC
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/assets/teaser-FX-football.xlsx
+++ b/docs/assets/teaser-FX-football.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Lisez-moi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs couverts'!$A$1:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs couverts'!$A$1:$N$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -455,12 +455,13 @@
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="62" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,20 +512,25 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>solde_mercato_2026_M_eur</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>volumes_fx_estimes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>nb_echeances_transfert</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>devises_principales</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>score_priorite</t>
         </is>
@@ -576,10 +582,8 @@
           <t>https://www.ol.fr/fr/actualites/ebury-devient-partenaire-fintech-de-l-olympique-lyonnais-pour-2025-2026</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
+      <c r="J2" t="n">
+        <v>44</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -592,6 +596,11 @@
         </is>
       </c>
       <c r="M2" t="inlineStr">
+        <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>non diffusé</t>
         </is>
@@ -643,10 +652,8 @@
           <t>https://www.asmonaco.com/en/news/ebury-new-fintech-partner-of-as-monaco</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
+      <c r="J3" t="n">
+        <v>56</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -659,6 +666,11 @@
         </is>
       </c>
       <c r="M3" t="inlineStr">
+        <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>non diffusé</t>
         </is>
@@ -710,10 +722,8 @@
           <t>https://www.asmonaco.com/en/news/sokin-nouveau-partenaire-officiel-de-las-monaco</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
+      <c r="J4" t="n">
+        <v>56</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -726,6 +736,11 @@
         </is>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>non diffusé</t>
         </is>
@@ -777,10 +792,8 @@
           <t>https://www.laprovence.com/article/economie/60019635627413/la-fintech-ebury-frappe-un-grand-coup-en-devenant-le-fournisseur-officiel-de-lolympique-de-marseille</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
+      <c r="J5" t="n">
+        <v>49.9</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -793,6 +806,11 @@
         </is>
       </c>
       <c r="M5" t="inlineStr">
+        <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>non diffusé</t>
         </is>
@@ -844,10 +862,8 @@
           <t>https://www.businesswire.com/news/home/20250220824657/fr</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
+      <c r="J6" t="n">
+        <v>25.5</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -860,6 +876,11 @@
         </is>
       </c>
       <c r="M6" t="inlineStr">
+        <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>non diffusé</t>
         </is>
@@ -911,11 +932,6 @@
           <t>https://www.stade-de-reims.com/ebury-devient-partenaire-premium-du-sdr/</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>non communiqué</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>non communiqué</t>
@@ -928,12 +944,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>non communiqué</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
           <t>non diffusé</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M7"/>
+  <autoFilter ref="A1:N7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -944,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1040,24 +1061,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Volumes FX par club</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>NON DIFFUSÉ</t>
+          <t>Soldes mercato été 2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Modèle interne, non publiable</t>
+          <t>Transfermarkt, relevés au 02/09/2026 (via Sportune / 20 Minutes)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Échéanciers de transfert</t>
+          <t>Volumes FX par club</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1074,49 +1095,66 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Devises par club</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PARTIEL</t>
+          <t>Échéanciers de transfert</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>NON DIFFUSÉ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Déduites des marchés de transfert, non vérifiées club par club</t>
+          <t>Modèle interne, non publiable</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Score de priorité commerciale</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>NON DIFFUSÉ</t>
+          <t>Devises par club</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PARTIEL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Résultat du scoring, non publiable</t>
+          <t>Déduites des marchés de transfert, non vérifiées club par club</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Score de priorité commerciale</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>NON DIFFUSÉ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Résultat du scoring, non publiable</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Noms d'entreprises / communes</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>NON DIFFUSÉ</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Conformément à la licence Orbis et par choix</t>
         </is>

</xml_diff>